<commit_message>
fix: swap dex and int growth in class table #928
- table: class ability dexterity and intelligence values swapped so each class grows its main stat
</commit_message>
<xml_diff>
--- a/resources/table/class.xlsx
+++ b/resources/table/class.xlsx
@@ -831,10 +831,10 @@
         <v>7</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>1</v>
@@ -854,10 +854,10 @@
         <v>8</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>1</v>
@@ -877,10 +877,10 @@
         <v>9</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>1</v>
@@ -969,10 +969,10 @@
         <v>13</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" s="7" t="n">
         <v>1</v>
@@ -992,10 +992,10 @@
         <v>14</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" s="7" t="n">
         <v>1</v>
@@ -1015,10 +1015,10 @@
         <v>15</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" s="7" t="n">
         <v>1</v>
@@ -1107,10 +1107,10 @@
         <v>19</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" s="7" t="n">
         <v>1</v>
@@ -1130,10 +1130,10 @@
         <v>20</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26" s="7" t="n">
         <v>1</v>
@@ -1153,10 +1153,10 @@
         <v>21</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" s="7" t="n">
         <v>1</v>
@@ -1245,10 +1245,10 @@
         <v>25</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D31" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>1</v>
@@ -1268,10 +1268,10 @@
         <v>26</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>1</v>
@@ -1291,10 +1291,10 @@
         <v>27</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D33" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" s="7" t="n">
         <v>1</v>
@@ -1383,10 +1383,10 @@
         <v>31</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D37" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E37" s="7" t="n">
         <v>1</v>
@@ -1406,10 +1406,10 @@
         <v>32</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>1</v>
@@ -1429,10 +1429,10 @@
         <v>33</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>1</v>
@@ -1521,10 +1521,10 @@
         <v>37</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D43" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E43" s="7" t="n">
         <v>1</v>
@@ -1544,10 +1544,10 @@
         <v>38</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D44" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" s="7" t="n">
         <v>1</v>
@@ -1567,10 +1567,10 @@
         <v>39</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D45" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E45" s="7" t="n">
         <v>1</v>
@@ -1659,10 +1659,10 @@
         <v>43</v>
       </c>
       <c r="C49" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D49" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E49" s="7" t="n">
         <v>1</v>
@@ -1682,10 +1682,10 @@
         <v>44</v>
       </c>
       <c r="C50" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D50" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E50" s="7" t="n">
         <v>1</v>
@@ -1705,10 +1705,10 @@
         <v>45</v>
       </c>
       <c r="C51" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D51" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E51" s="7" t="n">
         <v>1</v>
@@ -1797,10 +1797,10 @@
         <v>49</v>
       </c>
       <c r="C55" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D55" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E55" s="7" t="n">
         <v>1</v>
@@ -1820,10 +1820,10 @@
         <v>50</v>
       </c>
       <c r="C56" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D56" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E56" s="7" t="n">
         <v>1</v>
@@ -1843,10 +1843,10 @@
         <v>51</v>
       </c>
       <c r="C57" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D57" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E57" s="7" t="n">
         <v>1</v>
@@ -1935,10 +1935,10 @@
         <v>55</v>
       </c>
       <c r="C61" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D61" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E61" s="7" t="n">
         <v>1</v>
@@ -1958,10 +1958,10 @@
         <v>56</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E62" s="7" t="n">
         <v>1</v>
@@ -1981,10 +1981,10 @@
         <v>57</v>
       </c>
       <c r="C63" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D63" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E63" s="7" t="n">
         <v>1</v>
@@ -2073,10 +2073,10 @@
         <v>61</v>
       </c>
       <c r="C67" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D67" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E67" s="7" t="n">
         <v>1</v>
@@ -2096,10 +2096,10 @@
         <v>62</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E68" s="7" t="n">
         <v>1</v>
@@ -2119,10 +2119,10 @@
         <v>63</v>
       </c>
       <c r="C69" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D69" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E69" s="7" t="n">
         <v>1</v>
@@ -2211,10 +2211,10 @@
         <v>67</v>
       </c>
       <c r="C73" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D73" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E73" s="7" t="n">
         <v>1</v>
@@ -2234,10 +2234,10 @@
         <v>68</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E74" s="7" t="n">
         <v>1</v>
@@ -2257,10 +2257,10 @@
         <v>69</v>
       </c>
       <c r="C75" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D75" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E75" s="7" t="n">
         <v>1</v>
@@ -2349,10 +2349,10 @@
         <v>73</v>
       </c>
       <c r="C79" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D79" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E79" s="7" t="n">
         <v>1</v>
@@ -2372,10 +2372,10 @@
         <v>74</v>
       </c>
       <c r="C80" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E80" s="7" t="n">
         <v>1</v>
@@ -2395,10 +2395,10 @@
         <v>75</v>
       </c>
       <c r="C81" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E81" s="7" t="n">
         <v>1</v>
@@ -2487,10 +2487,10 @@
         <v>79</v>
       </c>
       <c r="C85" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D85" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E85" s="7" t="n">
         <v>1</v>
@@ -2510,10 +2510,10 @@
         <v>80</v>
       </c>
       <c r="C86" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D86" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E86" s="7" t="n">
         <v>1</v>
@@ -2533,10 +2533,10 @@
         <v>81</v>
       </c>
       <c r="C87" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D87" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E87" s="7" t="n">
         <v>1</v>
@@ -2625,10 +2625,10 @@
         <v>85</v>
       </c>
       <c r="C91" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D91" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E91" s="7" t="n">
         <v>1</v>
@@ -2648,10 +2648,10 @@
         <v>86</v>
       </c>
       <c r="C92" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D92" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E92" s="7" t="n">
         <v>1</v>
@@ -2671,10 +2671,10 @@
         <v>87</v>
       </c>
       <c r="C93" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D93" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E93" s="7" t="n">
         <v>1</v>
@@ -2763,10 +2763,10 @@
         <v>91</v>
       </c>
       <c r="C97" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D97" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E97" s="7" t="n">
         <v>1</v>
@@ -2786,10 +2786,10 @@
         <v>92</v>
       </c>
       <c r="C98" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D98" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E98" s="7" t="n">
         <v>1</v>
@@ -2809,10 +2809,10 @@
         <v>93</v>
       </c>
       <c r="C99" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D99" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E99" s="7" t="n">
         <v>1</v>
@@ -2901,10 +2901,10 @@
         <v>97</v>
       </c>
       <c r="C103" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D103" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E103" s="7" t="n">
         <v>1</v>
@@ -2924,10 +2924,10 @@
         <v>98</v>
       </c>
       <c r="C104" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D104" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E104" s="7" t="n">
         <v>1</v>
@@ -2947,10 +2947,10 @@
         <v>99</v>
       </c>
       <c r="C105" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D105" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E105" s="7" t="n">
         <v>1</v>
@@ -3008,10 +3008,10 @@
         <v>6</v>
       </c>
       <c r="C108" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D108" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E108" s="1" t="n">
         <v>0</v>
@@ -3056,10 +3056,10 @@
         <v>8</v>
       </c>
       <c r="C110" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D110" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E110" s="1" t="n">
         <v>1</v>
@@ -3104,10 +3104,10 @@
         <v>10</v>
       </c>
       <c r="C112" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D112" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E112" s="1" t="n">
         <v>0</v>
@@ -3152,10 +3152,10 @@
         <v>12</v>
       </c>
       <c r="C114" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D114" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E114" s="1" t="n">
         <v>0</v>
@@ -3200,10 +3200,10 @@
         <v>14</v>
       </c>
       <c r="C116" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D116" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E116" s="1" t="n">
         <v>1</v>
@@ -3248,10 +3248,10 @@
         <v>16</v>
       </c>
       <c r="C118" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D118" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E118" s="1" t="n">
         <v>0</v>
@@ -3296,10 +3296,10 @@
         <v>18</v>
       </c>
       <c r="C120" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D120" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E120" s="1" t="n">
         <v>0</v>
@@ -3344,10 +3344,10 @@
         <v>20</v>
       </c>
       <c r="C122" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D122" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E122" s="1" t="n">
         <v>1</v>
@@ -3392,10 +3392,10 @@
         <v>22</v>
       </c>
       <c r="C124" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D124" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E124" s="1" t="n">
         <v>0</v>
@@ -3440,10 +3440,10 @@
         <v>24</v>
       </c>
       <c r="C126" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D126" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E126" s="1" t="n">
         <v>0</v>
@@ -3488,10 +3488,10 @@
         <v>26</v>
       </c>
       <c r="C128" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D128" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E128" s="1" t="n">
         <v>1</v>
@@ -3536,10 +3536,10 @@
         <v>28</v>
       </c>
       <c r="C130" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D130" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E130" s="1" t="n">
         <v>0</v>
@@ -3584,10 +3584,10 @@
         <v>30</v>
       </c>
       <c r="C132" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D132" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E132" s="1" t="n">
         <v>0</v>
@@ -3632,10 +3632,10 @@
         <v>32</v>
       </c>
       <c r="C134" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D134" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E134" s="1" t="n">
         <v>1</v>
@@ -3680,10 +3680,10 @@
         <v>34</v>
       </c>
       <c r="C136" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D136" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E136" s="1" t="n">
         <v>0</v>
@@ -3728,10 +3728,10 @@
         <v>36</v>
       </c>
       <c r="C138" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D138" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E138" s="1" t="n">
         <v>0</v>
@@ -3776,10 +3776,10 @@
         <v>38</v>
       </c>
       <c r="C140" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D140" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E140" s="1" t="n">
         <v>1</v>
@@ -3824,10 +3824,10 @@
         <v>40</v>
       </c>
       <c r="C142" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D142" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E142" s="1" t="n">
         <v>0</v>
@@ -3872,10 +3872,10 @@
         <v>42</v>
       </c>
       <c r="C144" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D144" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E144" s="1" t="n">
         <v>0</v>
@@ -3920,10 +3920,10 @@
         <v>44</v>
       </c>
       <c r="C146" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D146" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E146" s="1" t="n">
         <v>1</v>
@@ -3968,10 +3968,10 @@
         <v>46</v>
       </c>
       <c r="C148" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D148" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E148" s="1" t="n">
         <v>0</v>
@@ -4016,10 +4016,10 @@
         <v>48</v>
       </c>
       <c r="C150" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D150" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E150" s="1" t="n">
         <v>0</v>
@@ -4064,10 +4064,10 @@
         <v>50</v>
       </c>
       <c r="C152" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D152" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E152" s="1" t="n">
         <v>1</v>
@@ -4112,10 +4112,10 @@
         <v>52</v>
       </c>
       <c r="C154" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D154" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E154" s="1" t="n">
         <v>0</v>
@@ -4160,10 +4160,10 @@
         <v>54</v>
       </c>
       <c r="C156" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D156" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E156" s="1" t="n">
         <v>0</v>
@@ -4208,10 +4208,10 @@
         <v>56</v>
       </c>
       <c r="C158" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D158" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E158" s="1" t="n">
         <v>1</v>
@@ -4256,10 +4256,10 @@
         <v>58</v>
       </c>
       <c r="C160" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D160" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E160" s="1" t="n">
         <v>0</v>
@@ -4304,10 +4304,10 @@
         <v>60</v>
       </c>
       <c r="C162" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D162" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E162" s="1" t="n">
         <v>0</v>
@@ -4352,10 +4352,10 @@
         <v>62</v>
       </c>
       <c r="C164" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D164" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E164" s="1" t="n">
         <v>1</v>
@@ -4400,10 +4400,10 @@
         <v>64</v>
       </c>
       <c r="C166" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D166" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E166" s="1" t="n">
         <v>0</v>
@@ -4448,10 +4448,10 @@
         <v>66</v>
       </c>
       <c r="C168" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D168" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E168" s="1" t="n">
         <v>0</v>
@@ -4496,10 +4496,10 @@
         <v>68</v>
       </c>
       <c r="C170" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D170" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E170" s="1" t="n">
         <v>1</v>
@@ -4544,10 +4544,10 @@
         <v>70</v>
       </c>
       <c r="C172" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D172" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E172" s="1" t="n">
         <v>0</v>
@@ -4592,10 +4592,10 @@
         <v>72</v>
       </c>
       <c r="C174" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D174" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E174" s="1" t="n">
         <v>0</v>
@@ -4640,10 +4640,10 @@
         <v>74</v>
       </c>
       <c r="C176" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D176" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E176" s="1" t="n">
         <v>1</v>
@@ -4688,10 +4688,10 @@
         <v>76</v>
       </c>
       <c r="C178" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D178" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E178" s="1" t="n">
         <v>0</v>
@@ -4736,10 +4736,10 @@
         <v>78</v>
       </c>
       <c r="C180" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D180" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E180" s="1" t="n">
         <v>0</v>
@@ -4784,10 +4784,10 @@
         <v>80</v>
       </c>
       <c r="C182" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D182" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E182" s="1" t="n">
         <v>1</v>
@@ -4832,10 +4832,10 @@
         <v>82</v>
       </c>
       <c r="C184" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D184" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E184" s="1" t="n">
         <v>0</v>
@@ -4880,10 +4880,10 @@
         <v>84</v>
       </c>
       <c r="C186" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D186" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E186" s="1" t="n">
         <v>0</v>
@@ -4928,10 +4928,10 @@
         <v>86</v>
       </c>
       <c r="C188" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D188" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E188" s="1" t="n">
         <v>1</v>
@@ -4976,10 +4976,10 @@
         <v>88</v>
       </c>
       <c r="C190" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D190" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E190" s="1" t="n">
         <v>0</v>
@@ -5024,10 +5024,10 @@
         <v>90</v>
       </c>
       <c r="C192" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D192" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E192" s="1" t="n">
         <v>0</v>
@@ -5072,10 +5072,10 @@
         <v>92</v>
       </c>
       <c r="C194" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D194" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E194" s="1" t="n">
         <v>1</v>
@@ -5120,10 +5120,10 @@
         <v>94</v>
       </c>
       <c r="C196" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D196" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E196" s="1" t="n">
         <v>0</v>
@@ -5168,10 +5168,10 @@
         <v>96</v>
       </c>
       <c r="C198" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D198" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E198" s="1" t="n">
         <v>0</v>
@@ -5216,10 +5216,10 @@
         <v>98</v>
       </c>
       <c r="C200" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D200" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E200" s="1" t="n">
         <v>1</v>
@@ -5278,10 +5278,10 @@
         <v>5</v>
       </c>
       <c r="C203" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D203" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E203" s="1" t="n">
         <v>0</v>
@@ -5302,10 +5302,10 @@
         <v>6</v>
       </c>
       <c r="C204" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D204" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E204" s="1" t="n">
         <v>0</v>
@@ -5350,10 +5350,10 @@
         <v>8</v>
       </c>
       <c r="C206" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D206" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E206" s="1" t="n">
         <v>0</v>
@@ -5398,10 +5398,10 @@
         <v>10</v>
       </c>
       <c r="C208" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D208" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E208" s="1" t="n">
         <v>0</v>
@@ -5422,10 +5422,10 @@
         <v>11</v>
       </c>
       <c r="C209" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D209" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E209" s="1" t="n">
         <v>0</v>
@@ -5470,10 +5470,10 @@
         <v>13</v>
       </c>
       <c r="C211" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D211" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E211" s="1" t="n">
         <v>0</v>
@@ -5518,10 +5518,10 @@
         <v>15</v>
       </c>
       <c r="C213" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D213" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E213" s="1" t="n">
         <v>0</v>
@@ -5542,10 +5542,10 @@
         <v>16</v>
       </c>
       <c r="C214" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D214" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E214" s="1" t="n">
         <v>0</v>
@@ -5590,10 +5590,10 @@
         <v>18</v>
       </c>
       <c r="C216" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D216" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E216" s="1" t="n">
         <v>0</v>
@@ -5638,10 +5638,10 @@
         <v>20</v>
       </c>
       <c r="C218" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D218" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E218" s="1" t="n">
         <v>0</v>
@@ -5662,10 +5662,10 @@
         <v>21</v>
       </c>
       <c r="C219" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D219" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E219" s="1" t="n">
         <v>0</v>
@@ -5710,10 +5710,10 @@
         <v>23</v>
       </c>
       <c r="C221" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D221" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E221" s="1" t="n">
         <v>0</v>
@@ -5758,10 +5758,10 @@
         <v>25</v>
       </c>
       <c r="C223" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D223" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E223" s="1" t="n">
         <v>0</v>
@@ -5782,10 +5782,10 @@
         <v>26</v>
       </c>
       <c r="C224" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D224" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E224" s="1" t="n">
         <v>0</v>
@@ -5830,10 +5830,10 @@
         <v>28</v>
       </c>
       <c r="C226" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D226" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E226" s="1" t="n">
         <v>0</v>
@@ -5878,10 +5878,10 @@
         <v>30</v>
       </c>
       <c r="C228" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D228" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E228" s="1" t="n">
         <v>0</v>
@@ -5902,10 +5902,10 @@
         <v>31</v>
       </c>
       <c r="C229" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D229" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E229" s="1" t="n">
         <v>0</v>
@@ -5950,10 +5950,10 @@
         <v>33</v>
       </c>
       <c r="C231" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D231" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E231" s="1" t="n">
         <v>0</v>
@@ -5998,10 +5998,10 @@
         <v>35</v>
       </c>
       <c r="C233" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D233" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E233" s="1" t="n">
         <v>0</v>
@@ -6022,10 +6022,10 @@
         <v>36</v>
       </c>
       <c r="C234" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D234" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E234" s="1" t="n">
         <v>0</v>
@@ -6070,10 +6070,10 @@
         <v>38</v>
       </c>
       <c r="C236" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D236" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E236" s="1" t="n">
         <v>0</v>
@@ -6118,10 +6118,10 @@
         <v>40</v>
       </c>
       <c r="C238" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D238" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E238" s="1" t="n">
         <v>0</v>
@@ -6142,10 +6142,10 @@
         <v>41</v>
       </c>
       <c r="C239" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D239" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E239" s="1" t="n">
         <v>0</v>
@@ -6190,10 +6190,10 @@
         <v>43</v>
       </c>
       <c r="C241" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D241" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E241" s="1" t="n">
         <v>0</v>
@@ -6238,10 +6238,10 @@
         <v>45</v>
       </c>
       <c r="C243" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D243" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E243" s="1" t="n">
         <v>0</v>
@@ -6262,10 +6262,10 @@
         <v>46</v>
       </c>
       <c r="C244" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D244" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E244" s="1" t="n">
         <v>0</v>
@@ -6310,10 +6310,10 @@
         <v>48</v>
       </c>
       <c r="C246" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D246" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E246" s="1" t="n">
         <v>0</v>
@@ -6358,10 +6358,10 @@
         <v>50</v>
       </c>
       <c r="C248" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D248" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E248" s="1" t="n">
         <v>0</v>
@@ -6382,10 +6382,10 @@
         <v>51</v>
       </c>
       <c r="C249" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D249" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E249" s="1" t="n">
         <v>0</v>
@@ -6430,10 +6430,10 @@
         <v>53</v>
       </c>
       <c r="C251" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D251" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E251" s="1" t="n">
         <v>0</v>
@@ -6478,10 +6478,10 @@
         <v>55</v>
       </c>
       <c r="C253" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D253" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E253" s="1" t="n">
         <v>0</v>
@@ -6502,10 +6502,10 @@
         <v>56</v>
       </c>
       <c r="C254" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D254" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E254" s="1" t="n">
         <v>0</v>
@@ -6550,10 +6550,10 @@
         <v>58</v>
       </c>
       <c r="C256" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D256" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E256" s="1" t="n">
         <v>0</v>
@@ -6598,10 +6598,10 @@
         <v>60</v>
       </c>
       <c r="C258" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D258" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E258" s="1" t="n">
         <v>0</v>
@@ -6622,10 +6622,10 @@
         <v>61</v>
       </c>
       <c r="C259" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D259" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E259" s="1" t="n">
         <v>0</v>
@@ -6670,10 +6670,10 @@
         <v>63</v>
       </c>
       <c r="C261" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D261" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E261" s="1" t="n">
         <v>0</v>
@@ -6718,10 +6718,10 @@
         <v>65</v>
       </c>
       <c r="C263" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D263" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E263" s="1" t="n">
         <v>0</v>
@@ -6742,10 +6742,10 @@
         <v>66</v>
       </c>
       <c r="C264" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D264" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E264" s="1" t="n">
         <v>0</v>
@@ -6790,10 +6790,10 @@
         <v>68</v>
       </c>
       <c r="C266" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D266" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E266" s="1" t="n">
         <v>0</v>
@@ -6838,10 +6838,10 @@
         <v>70</v>
       </c>
       <c r="C268" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D268" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E268" s="1" t="n">
         <v>0</v>
@@ -6862,10 +6862,10 @@
         <v>71</v>
       </c>
       <c r="C269" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D269" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E269" s="1" t="n">
         <v>0</v>
@@ -6910,10 +6910,10 @@
         <v>73</v>
       </c>
       <c r="C271" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D271" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E271" s="1" t="n">
         <v>0</v>
@@ -6958,10 +6958,10 @@
         <v>75</v>
       </c>
       <c r="C273" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D273" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E273" s="1" t="n">
         <v>0</v>
@@ -6982,10 +6982,10 @@
         <v>76</v>
       </c>
       <c r="C274" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D274" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E274" s="1" t="n">
         <v>0</v>
@@ -7030,10 +7030,10 @@
         <v>78</v>
       </c>
       <c r="C276" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D276" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E276" s="1" t="n">
         <v>0</v>
@@ -7078,10 +7078,10 @@
         <v>80</v>
       </c>
       <c r="C278" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D278" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E278" s="1" t="n">
         <v>0</v>
@@ -7102,10 +7102,10 @@
         <v>81</v>
       </c>
       <c r="C279" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D279" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E279" s="1" t="n">
         <v>0</v>
@@ -7150,10 +7150,10 @@
         <v>83</v>
       </c>
       <c r="C281" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D281" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E281" s="1" t="n">
         <v>0</v>
@@ -7198,10 +7198,10 @@
         <v>85</v>
       </c>
       <c r="C283" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D283" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E283" s="1" t="n">
         <v>0</v>
@@ -7222,10 +7222,10 @@
         <v>86</v>
       </c>
       <c r="C284" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D284" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E284" s="1" t="n">
         <v>0</v>
@@ -7270,10 +7270,10 @@
         <v>88</v>
       </c>
       <c r="C286" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D286" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E286" s="1" t="n">
         <v>0</v>
@@ -7318,10 +7318,10 @@
         <v>90</v>
       </c>
       <c r="C288" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D288" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E288" s="1" t="n">
         <v>0</v>
@@ -7342,10 +7342,10 @@
         <v>91</v>
       </c>
       <c r="C289" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D289" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E289" s="1" t="n">
         <v>0</v>
@@ -7390,10 +7390,10 @@
         <v>93</v>
       </c>
       <c r="C291" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D291" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E291" s="1" t="n">
         <v>0</v>
@@ -7438,10 +7438,10 @@
         <v>95</v>
       </c>
       <c r="C293" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D293" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E293" s="1" t="n">
         <v>0</v>
@@ -7462,10 +7462,10 @@
         <v>96</v>
       </c>
       <c r="C294" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D294" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E294" s="1" t="n">
         <v>0</v>
@@ -7510,10 +7510,10 @@
         <v>98</v>
       </c>
       <c r="C296" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D296" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E296" s="1" t="n">
         <v>0</v>
@@ -7596,10 +7596,10 @@
         <v>6</v>
       </c>
       <c r="C300" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D300" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E300" s="1" t="n">
         <v>0</v>
@@ -7644,10 +7644,10 @@
         <v>8</v>
       </c>
       <c r="C302" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D302" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E302" s="1" t="n">
         <v>0</v>
@@ -7668,10 +7668,10 @@
         <v>9</v>
       </c>
       <c r="C303" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D303" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E303" s="1" t="n">
         <v>0</v>
@@ -7716,10 +7716,10 @@
         <v>11</v>
       </c>
       <c r="C305" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D305" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E305" s="1" t="n">
         <v>0</v>
@@ -7740,10 +7740,10 @@
         <v>12</v>
       </c>
       <c r="C306" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D306" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E306" s="1" t="n">
         <v>0</v>
@@ -7788,10 +7788,10 @@
         <v>14</v>
       </c>
       <c r="C308" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D308" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E308" s="1" t="n">
         <v>0</v>
@@ -7836,10 +7836,10 @@
         <v>16</v>
       </c>
       <c r="C310" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D310" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E310" s="1" t="n">
         <v>0</v>
@@ -7860,10 +7860,10 @@
         <v>17</v>
       </c>
       <c r="C311" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D311" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E311" s="1" t="n">
         <v>0</v>
@@ -7908,10 +7908,10 @@
         <v>19</v>
       </c>
       <c r="C313" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D313" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E313" s="1" t="n">
         <v>0</v>
@@ -7932,10 +7932,10 @@
         <v>20</v>
       </c>
       <c r="C314" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D314" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E314" s="1" t="n">
         <v>0</v>
@@ -7980,10 +7980,10 @@
         <v>22</v>
       </c>
       <c r="C316" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D316" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E316" s="1" t="n">
         <v>0</v>
@@ -8028,10 +8028,10 @@
         <v>24</v>
       </c>
       <c r="C318" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D318" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E318" s="1" t="n">
         <v>0</v>
@@ -8052,10 +8052,10 @@
         <v>25</v>
       </c>
       <c r="C319" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D319" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E319" s="1" t="n">
         <v>0</v>
@@ -8100,10 +8100,10 @@
         <v>27</v>
       </c>
       <c r="C321" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D321" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E321" s="1" t="n">
         <v>0</v>
@@ -8124,10 +8124,10 @@
         <v>28</v>
       </c>
       <c r="C322" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D322" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E322" s="1" t="n">
         <v>0</v>
@@ -8172,10 +8172,10 @@
         <v>30</v>
       </c>
       <c r="C324" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D324" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E324" s="1" t="n">
         <v>0</v>
@@ -8220,10 +8220,10 @@
         <v>32</v>
       </c>
       <c r="C326" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D326" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E326" s="1" t="n">
         <v>0</v>
@@ -8244,10 +8244,10 @@
         <v>33</v>
       </c>
       <c r="C327" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D327" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E327" s="1" t="n">
         <v>0</v>
@@ -8292,10 +8292,10 @@
         <v>35</v>
       </c>
       <c r="C329" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D329" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E329" s="1" t="n">
         <v>0</v>
@@ -8316,10 +8316,10 @@
         <v>36</v>
       </c>
       <c r="C330" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D330" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E330" s="1" t="n">
         <v>0</v>
@@ -8364,10 +8364,10 @@
         <v>38</v>
       </c>
       <c r="C332" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D332" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E332" s="1" t="n">
         <v>0</v>
@@ -8412,10 +8412,10 @@
         <v>40</v>
       </c>
       <c r="C334" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D334" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E334" s="1" t="n">
         <v>0</v>
@@ -8436,10 +8436,10 @@
         <v>41</v>
       </c>
       <c r="C335" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D335" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E335" s="1" t="n">
         <v>0</v>
@@ -8484,10 +8484,10 @@
         <v>43</v>
       </c>
       <c r="C337" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D337" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E337" s="1" t="n">
         <v>0</v>
@@ -8508,10 +8508,10 @@
         <v>44</v>
       </c>
       <c r="C338" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D338" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E338" s="1" t="n">
         <v>0</v>
@@ -8556,10 +8556,10 @@
         <v>46</v>
       </c>
       <c r="C340" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D340" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E340" s="1" t="n">
         <v>0</v>
@@ -8604,10 +8604,10 @@
         <v>48</v>
       </c>
       <c r="C342" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D342" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E342" s="1" t="n">
         <v>0</v>
@@ -8628,10 +8628,10 @@
         <v>49</v>
       </c>
       <c r="C343" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D343" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E343" s="1" t="n">
         <v>0</v>
@@ -8676,10 +8676,10 @@
         <v>51</v>
       </c>
       <c r="C345" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D345" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E345" s="1" t="n">
         <v>0</v>
@@ -8700,10 +8700,10 @@
         <v>52</v>
       </c>
       <c r="C346" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D346" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E346" s="1" t="n">
         <v>0</v>
@@ -8748,10 +8748,10 @@
         <v>54</v>
       </c>
       <c r="C348" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D348" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E348" s="1" t="n">
         <v>0</v>
@@ -8796,10 +8796,10 @@
         <v>56</v>
       </c>
       <c r="C350" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D350" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E350" s="1" t="n">
         <v>0</v>
@@ -8820,10 +8820,10 @@
         <v>57</v>
       </c>
       <c r="C351" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D351" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E351" s="1" t="n">
         <v>0</v>
@@ -8868,10 +8868,10 @@
         <v>59</v>
       </c>
       <c r="C353" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D353" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E353" s="1" t="n">
         <v>0</v>
@@ -8892,10 +8892,10 @@
         <v>60</v>
       </c>
       <c r="C354" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D354" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E354" s="1" t="n">
         <v>0</v>
@@ -8940,10 +8940,10 @@
         <v>62</v>
       </c>
       <c r="C356" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D356" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E356" s="1" t="n">
         <v>0</v>
@@ -8988,10 +8988,10 @@
         <v>64</v>
       </c>
       <c r="C358" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D358" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E358" s="1" t="n">
         <v>0</v>
@@ -9012,10 +9012,10 @@
         <v>65</v>
       </c>
       <c r="C359" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D359" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E359" s="1" t="n">
         <v>0</v>
@@ -9060,10 +9060,10 @@
         <v>67</v>
       </c>
       <c r="C361" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D361" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E361" s="1" t="n">
         <v>0</v>
@@ -9084,10 +9084,10 @@
         <v>68</v>
       </c>
       <c r="C362" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D362" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E362" s="1" t="n">
         <v>0</v>
@@ -9132,10 +9132,10 @@
         <v>70</v>
       </c>
       <c r="C364" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D364" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E364" s="1" t="n">
         <v>0</v>
@@ -9180,10 +9180,10 @@
         <v>72</v>
       </c>
       <c r="C366" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D366" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E366" s="1" t="n">
         <v>0</v>
@@ -9204,10 +9204,10 @@
         <v>73</v>
       </c>
       <c r="C367" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D367" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E367" s="1" t="n">
         <v>0</v>
@@ -9252,10 +9252,10 @@
         <v>75</v>
       </c>
       <c r="C369" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D369" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E369" s="1" t="n">
         <v>0</v>
@@ -9276,10 +9276,10 @@
         <v>76</v>
       </c>
       <c r="C370" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D370" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E370" s="1" t="n">
         <v>0</v>
@@ -9324,10 +9324,10 @@
         <v>78</v>
       </c>
       <c r="C372" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D372" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E372" s="1" t="n">
         <v>0</v>
@@ -9372,10 +9372,10 @@
         <v>80</v>
       </c>
       <c r="C374" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D374" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E374" s="1" t="n">
         <v>0</v>
@@ -9396,10 +9396,10 @@
         <v>81</v>
       </c>
       <c r="C375" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D375" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E375" s="1" t="n">
         <v>0</v>
@@ -9444,10 +9444,10 @@
         <v>83</v>
       </c>
       <c r="C377" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D377" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E377" s="1" t="n">
         <v>0</v>
@@ -9468,10 +9468,10 @@
         <v>84</v>
       </c>
       <c r="C378" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D378" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E378" s="1" t="n">
         <v>0</v>
@@ -9516,10 +9516,10 @@
         <v>86</v>
       </c>
       <c r="C380" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D380" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E380" s="1" t="n">
         <v>0</v>
@@ -9564,10 +9564,10 @@
         <v>88</v>
       </c>
       <c r="C382" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D382" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E382" s="1" t="n">
         <v>0</v>
@@ -9588,10 +9588,10 @@
         <v>89</v>
       </c>
       <c r="C383" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D383" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E383" s="1" t="n">
         <v>0</v>
@@ -9636,10 +9636,10 @@
         <v>91</v>
       </c>
       <c r="C385" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D385" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E385" s="1" t="n">
         <v>0</v>
@@ -9660,10 +9660,10 @@
         <v>92</v>
       </c>
       <c r="C386" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D386" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E386" s="1" t="n">
         <v>0</v>
@@ -9708,10 +9708,10 @@
         <v>94</v>
       </c>
       <c r="C388" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D388" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E388" s="1" t="n">
         <v>0</v>
@@ -9756,10 +9756,10 @@
         <v>96</v>
       </c>
       <c r="C390" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D390" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E390" s="1" t="n">
         <v>0</v>
@@ -9780,10 +9780,10 @@
         <v>97</v>
       </c>
       <c r="C391" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D391" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E391" s="1" t="n">
         <v>0</v>
@@ -9828,10 +9828,10 @@
         <v>99</v>
       </c>
       <c r="C393" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D393" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E393" s="1" t="n">
         <v>0</v>

</xml_diff>